<commit_message>
tambah download excel di halaman evaluasi
</commit_message>
<xml_diff>
--- a/penilaian-ZI.xlsx
+++ b/penilaian-ZI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\project\sibekisar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEFF3CD2-0BC7-4CE9-8D97-107C3DB945B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC22B74-640C-4B20-B0A7-D15D4E9E7224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{81ABB71F-C48B-4169-A963-AC8D91DB89DC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{81ABB71F-C48B-4169-A963-AC8D91DB89DC}"/>
   </bookViews>
   <sheets>
     <sheet name="RB General" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2721" uniqueCount="740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2713" uniqueCount="763">
   <si>
     <t>Indikator</t>
   </si>
@@ -2260,6 +2260,75 @@
   </si>
   <si>
     <t>insert into m_indikator (id_indikator,indikator,id_aspek,bobot,nilai_maks,periode,jml_periode,opd_pengampu,id_opd,tag,keterangan,is_aktif) values</t>
+  </si>
+  <si>
+    <t>C0202503</t>
+  </si>
+  <si>
+    <t>C020250301</t>
+  </si>
+  <si>
+    <t>Rencana Aksi Pengentasan Kemiskinan</t>
+  </si>
+  <si>
+    <t>Rencana Aksi Realisasi Investasi</t>
+  </si>
+  <si>
+    <t>Rencana Aksi Mendorong Hilirisasi</t>
+  </si>
+  <si>
+    <t>Rencana Aksi Mendukung Ketahanan Pangan Nasional</t>
+  </si>
+  <si>
+    <t>Rencana Aksi Peningkatan Kualitas dan Akses Layanan Kesehatan</t>
+  </si>
+  <si>
+    <t>Rencana Aksi Peningkatan Akses, Kualitas dan Mutu Layanan Pendidikan</t>
+  </si>
+  <si>
+    <t>C020250304</t>
+  </si>
+  <si>
+    <t>C020250305</t>
+  </si>
+  <si>
+    <t>C020250306</t>
+  </si>
+  <si>
+    <t>C020250406</t>
+  </si>
+  <si>
+    <t>C0202504</t>
+  </si>
+  <si>
+    <t>C020250401</t>
+  </si>
+  <si>
+    <t>Capaian Output Pengentasan Kemiskinan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capaian Output Realisasi Investasi </t>
+  </si>
+  <si>
+    <t>Capaian Output Mendorong Hilirisasi</t>
+  </si>
+  <si>
+    <t>Capaian Output Mendukung Ketahanan Pangan Nasional</t>
+  </si>
+  <si>
+    <t>Capaian Output Peningkatan Kualitas dan Akses Layanan Kesehatan</t>
+  </si>
+  <si>
+    <t>Capaian Output Peningkatan Akses, Kualitas dan Mutu Layanan Pendidikan</t>
+  </si>
+  <si>
+    <t>C020250403</t>
+  </si>
+  <si>
+    <t>C020250405</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insert into m_indikator (id_indikator, indikator, id_aspek, bobot, nilai_maks, periode, jml_periode, opd_pengampu, id_opd, tag, keterangan, is_aktif) values </t>
   </si>
 </sst>
 </file>
@@ -2431,6 +2500,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2457,11 +2531,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2792,16 +2861,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="H1" s="19" t="s">
+      <c r="H1" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="I1" s="19"/>
+      <c r="I1" s="22"/>
     </row>
     <row r="2" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18"/>
+      <c r="C2" s="21"/>
       <c r="D2" s="4" t="s">
         <v>42</v>
       </c>
@@ -2819,21 +2888,21 @@
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B3" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="26"/>
+      <c r="B3" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="29"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="6">
         <f>SUM(F4:F7)</f>
         <v>10</v>
       </c>
-      <c r="H3" s="20">
+      <c r="H3" s="23">
         <f>SUM(I4:I7)</f>
         <v>8.8000000000000007</v>
       </c>
-      <c r="I3" s="21"/>
+      <c r="I3" s="24"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B4" s="7">
@@ -2932,21 +3001,21 @@
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="26"/>
+      <c r="C8" s="29"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="6">
         <f>SUM(F9:F38)</f>
         <v>100</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="23">
         <f>SUM(I9:I38)</f>
         <v>100</v>
       </c>
-      <c r="I8" s="21"/>
+      <c r="I8" s="24"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B9" s="7">
@@ -3669,12 +3738,12 @@
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B39" s="22" t="s">
+      <c r="B39" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C39" s="23"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="24"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="27"/>
       <c r="F39" s="9">
         <f>F3+F8</f>
         <v>110</v>
@@ -4440,11 +4509,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:13" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="27" t="s">
+    <row r="34" spans="1:13" s="19" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="18" t="s">
         <v>727</v>
       </c>
-      <c r="D34" s="29"/>
+      <c r="D34" s="20"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
@@ -28589,10 +28658,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CC0CF0B-7DF2-48BE-A9BA-1DAA62A1A90A}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -28600,190 +28674,387 @@
         <v>46</v>
       </c>
       <c r="C1" t="s">
-        <v>712</v>
+        <v>728</v>
       </c>
       <c r="D1" t="s">
-        <v>713</v>
+        <v>47</v>
       </c>
       <c r="E1" t="s">
         <v>48</v>
       </c>
       <c r="F1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+        <v>729</v>
+      </c>
+      <c r="G1" t="s">
+        <v>730</v>
+      </c>
+      <c r="H1" t="s">
+        <v>712</v>
+      </c>
+      <c r="I1" t="s">
+        <v>713</v>
+      </c>
+      <c r="J1" t="s">
+        <v>731</v>
+      </c>
+      <c r="K1" t="s">
+        <v>732</v>
+      </c>
+      <c r="L1" t="s">
+        <v>733</v>
+      </c>
+      <c r="M1" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>741</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>742</v>
       </c>
       <c r="C2" t="s">
-        <v>714</v>
+        <v>740</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="F2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>715</v>
+      </c>
+      <c r="I2">
+        <v>55</v>
+      </c>
+      <c r="J2" t="s">
+        <v>734</v>
+      </c>
+      <c r="K2" t="s">
+        <v>715</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="str">
+        <f>"('"&amp;A2&amp;"', '"&amp;B2&amp;"', '"&amp;C2&amp;"', "&amp;D2&amp;", "&amp;E2&amp;", "&amp;F2&amp;", "&amp;G2&amp;", '"&amp;H2&amp;"', "&amp;I2&amp;", '"&amp;J2&amp;"', '"&amp;K2&amp;"', "&amp;L2&amp;"),"</f>
+        <v>('C020250301', 'Rencana Aksi Pengentasan Kemiskinan', 'C0202503', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>743</v>
       </c>
       <c r="C3" t="s">
+        <v>740</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
         <v>715</v>
       </c>
-      <c r="D3">
+      <c r="I3">
         <v>55</v>
       </c>
-      <c r="E3">
-        <v>100</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="J3" t="s">
+        <v>734</v>
+      </c>
+      <c r="K3" t="s">
+        <v>715</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="str">
+        <f t="shared" ref="M3:M13" si="0">"('"&amp;A3&amp;"', '"&amp;B3&amp;"', '"&amp;C3&amp;"', "&amp;D3&amp;", "&amp;E3&amp;", "&amp;F3&amp;", "&amp;G3&amp;", '"&amp;H3&amp;"', "&amp;I3&amp;", '"&amp;J3&amp;"', '"&amp;K3&amp;"', "&amp;L3&amp;"),"</f>
+        <v>('C020250302', 'Rencana Aksi Realisasi Investasi', 'C0202503', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>179</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>744</v>
       </c>
       <c r="C4" t="s">
-        <v>714</v>
+        <v>740</v>
       </c>
       <c r="D4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>100</v>
       </c>
       <c r="F4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>715</v>
+      </c>
+      <c r="I4">
+        <v>55</v>
+      </c>
+      <c r="J4" t="s">
+        <v>734</v>
+      </c>
+      <c r="K4" t="s">
+        <v>715</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250303', 'Rencana Aksi Mendorong Hilirisasi', 'C0202503', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>748</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>745</v>
       </c>
       <c r="C5" t="s">
-        <v>717</v>
+        <v>740</v>
       </c>
       <c r="D5">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>100</v>
       </c>
       <c r="F5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>715</v>
+      </c>
+      <c r="I5">
+        <v>55</v>
+      </c>
+      <c r="J5" t="s">
+        <v>734</v>
+      </c>
+      <c r="K5" t="s">
+        <v>715</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250304', 'Rencana Aksi Mendukung Ketahanan Pangan Nasional', 'C0202503', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>749</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>746</v>
       </c>
       <c r="C6" t="s">
-        <v>717</v>
+        <v>740</v>
       </c>
       <c r="D6">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="E6">
         <v>100</v>
       </c>
       <c r="F6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>715</v>
+      </c>
+      <c r="I6">
+        <v>55</v>
+      </c>
+      <c r="J6" t="s">
+        <v>734</v>
+      </c>
+      <c r="K6" t="s">
+        <v>715</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250305', 'Rencana Aksi Peningkatan Kualitas dan Akses Layanan Kesehatan', 'C0202503', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>750</v>
+      </c>
+      <c r="B7" t="s">
+        <v>747</v>
+      </c>
+      <c r="C7" t="s">
+        <v>740</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>100</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>715</v>
+      </c>
+      <c r="I7">
         <v>55</v>
       </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" t="s">
-        <v>718</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>100</v>
-      </c>
-      <c r="F7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="J7" t="s">
+        <v>734</v>
+      </c>
+      <c r="K7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250306', 'Rencana Aksi Peningkatan Akses, Kualitas dan Mutu Layanan Pendidikan', 'C0202503', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>753</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>754</v>
       </c>
       <c r="C8" t="s">
-        <v>719</v>
+        <v>752</v>
       </c>
       <c r="D8">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="E8">
         <v>100</v>
       </c>
       <c r="F8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>715</v>
+      </c>
+      <c r="I8">
+        <v>55</v>
+      </c>
+      <c r="J8" t="s">
+        <v>734</v>
+      </c>
+      <c r="K8" t="s">
+        <v>715</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250401', 'Capaian Output Pengentasan Kemiskinan', 'C0202504', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>244</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>755</v>
       </c>
       <c r="C9" t="s">
-        <v>719</v>
+        <v>752</v>
       </c>
       <c r="D9">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="E9">
         <v>100</v>
       </c>
       <c r="F9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>715</v>
+      </c>
+      <c r="I9">
+        <v>55</v>
+      </c>
+      <c r="J9" t="s">
+        <v>734</v>
+      </c>
+      <c r="K9" t="s">
+        <v>715</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250402', 'Capaian Output Realisasi Investasi ', 'C0202504', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>760</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>756</v>
       </c>
       <c r="C10" t="s">
-        <v>719</v>
+        <v>752</v>
       </c>
       <c r="D10">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="E10">
         <v>100</v>
@@ -28791,408 +29062,158 @@
       <c r="F10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>715</v>
+      </c>
+      <c r="I10">
+        <v>55</v>
+      </c>
+      <c r="J10" t="s">
+        <v>734</v>
+      </c>
+      <c r="K10" t="s">
+        <v>715</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250403', 'Capaian Output Mendorong Hilirisasi', 'C0202504', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>309</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>757</v>
       </c>
       <c r="C11" t="s">
-        <v>719</v>
+        <v>752</v>
       </c>
       <c r="D11">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>100</v>
       </c>
       <c r="F11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11" t="s">
+        <v>715</v>
+      </c>
+      <c r="I11">
+        <v>55</v>
+      </c>
+      <c r="J11" t="s">
+        <v>734</v>
+      </c>
+      <c r="K11" t="s">
+        <v>715</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250404', 'Capaian Output Mendukung Ketahanan Pangan Nasional', 'C0202504', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>761</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>758</v>
       </c>
       <c r="C12" t="s">
-        <v>719</v>
+        <v>752</v>
       </c>
       <c r="D12">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="E12">
         <v>100</v>
       </c>
       <c r="F12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12" t="s">
+        <v>715</v>
+      </c>
+      <c r="I12">
+        <v>55</v>
+      </c>
+      <c r="J12" t="s">
+        <v>734</v>
+      </c>
+      <c r="K12" t="s">
+        <v>715</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250405', 'Capaian Output Peningkatan Kualitas dan Akses Layanan Kesehatan', 'C0202504', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>751</v>
       </c>
       <c r="B13" t="s">
-        <v>711</v>
+        <v>759</v>
       </c>
       <c r="C13" t="s">
-        <v>720</v>
+        <v>752</v>
       </c>
       <c r="D13">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E13">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="F13">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13" t="s">
         <v>715</v>
       </c>
-      <c r="D14">
+      <c r="I13">
         <v>55</v>
       </c>
-      <c r="E14">
-        <v>100</v>
-      </c>
-      <c r="F14">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" t="s">
-        <v>724</v>
-      </c>
-      <c r="D15">
-        <v>31</v>
-      </c>
-      <c r="E15">
-        <v>100</v>
-      </c>
-      <c r="F15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>65</v>
-      </c>
-      <c r="B16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" t="s">
-        <v>720</v>
-      </c>
-      <c r="D16">
-        <v>21</v>
-      </c>
-      <c r="E16">
-        <v>100</v>
-      </c>
-      <c r="F16">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>66</v>
-      </c>
-      <c r="B17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" t="s">
-        <v>720</v>
-      </c>
-      <c r="D17">
-        <v>21</v>
-      </c>
-      <c r="E17">
-        <v>100</v>
-      </c>
-      <c r="F17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" t="s">
-        <v>719</v>
-      </c>
-      <c r="D18">
-        <v>52</v>
-      </c>
-      <c r="E18">
-        <v>100</v>
-      </c>
-      <c r="F18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>68</v>
-      </c>
-      <c r="B19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" t="s">
-        <v>721</v>
-      </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
-      <c r="E19">
-        <v>100</v>
-      </c>
-      <c r="F19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B20" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20" t="s">
-        <v>720</v>
-      </c>
-      <c r="D20">
-        <v>21</v>
-      </c>
-      <c r="E20">
-        <v>100</v>
-      </c>
-      <c r="F20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>71</v>
-      </c>
-      <c r="B21" t="s">
-        <v>72</v>
-      </c>
-      <c r="C21" t="s">
-        <v>720</v>
-      </c>
-      <c r="D21">
-        <v>21</v>
-      </c>
-      <c r="E21">
-        <v>100</v>
-      </c>
-      <c r="F21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>73</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="J13" t="s">
+        <v>734</v>
+      </c>
+      <c r="K13" t="s">
         <v>715</v>
       </c>
-      <c r="D22">
-        <v>55</v>
-      </c>
-      <c r="E22">
-        <v>100</v>
-      </c>
-      <c r="F22">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>74</v>
-      </c>
-      <c r="B23" t="s">
-        <v>30</v>
-      </c>
-      <c r="C23" t="s">
-        <v>715</v>
-      </c>
-      <c r="D23">
-        <v>55</v>
-      </c>
-      <c r="E23">
-        <v>100</v>
-      </c>
-      <c r="F23">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>75</v>
-      </c>
-      <c r="B24" t="s">
-        <v>31</v>
-      </c>
-      <c r="C24" t="s">
-        <v>722</v>
-      </c>
-      <c r="D24">
-        <v>39</v>
-      </c>
-      <c r="E24">
-        <v>100</v>
-      </c>
-      <c r="F24">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>77</v>
-      </c>
-      <c r="B25" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" t="s">
-        <v>716</v>
-      </c>
-      <c r="D25">
-        <v>6</v>
-      </c>
-      <c r="E25">
-        <v>4</v>
-      </c>
-      <c r="F25">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>79</v>
-      </c>
-      <c r="B26" t="s">
-        <v>725</v>
-      </c>
-      <c r="C26" t="s">
-        <v>715</v>
-      </c>
-      <c r="D26">
-        <v>55</v>
-      </c>
-      <c r="E26">
-        <v>100</v>
-      </c>
-      <c r="F26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>81</v>
-      </c>
-      <c r="B27" t="s">
-        <v>34</v>
-      </c>
-      <c r="C27" t="s">
-        <v>721</v>
-      </c>
-      <c r="D27">
-        <v>1</v>
-      </c>
-      <c r="E27">
-        <v>100</v>
-      </c>
-      <c r="F27">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>82</v>
-      </c>
-      <c r="B28" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" t="s">
-        <v>723</v>
-      </c>
-      <c r="D28">
-        <v>7</v>
-      </c>
-      <c r="E28">
-        <v>100</v>
-      </c>
-      <c r="F28">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>83</v>
-      </c>
-      <c r="B29" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" t="s">
-        <v>720</v>
-      </c>
-      <c r="D29">
-        <v>21</v>
-      </c>
-      <c r="E29">
-        <v>100</v>
-      </c>
-      <c r="F29">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>84</v>
-      </c>
-      <c r="B30" t="s">
-        <v>37</v>
-      </c>
-      <c r="C30" t="s">
-        <v>720</v>
-      </c>
-      <c r="D30">
-        <v>21</v>
-      </c>
-      <c r="E30">
-        <v>5</v>
-      </c>
-      <c r="F30">
-        <v>3</v>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="str">
+        <f t="shared" si="0"/>
+        <v>('C020250406', 'Capaian Output Peningkatan Akses, Kualitas dan Mutu Layanan Pendidikan', 'C0202504', 1, 100, 1, 1, 'Biro Organisasi', 55, 'opd', 'Biro Organisasi', 1),</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>